<commit_message>
Update mysql2 and deployment fixes
</commit_message>
<xml_diff>
--- a/backend/payments.xlsx
+++ b/backend/payments.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="482">
   <si>
     <t>Date</t>
   </si>
@@ -1361,6 +1361,102 @@
   </si>
   <si>
     <t>vgyhg</t>
+  </si>
+  <si>
+    <t>27/10/2025, 11:06:31 pm</t>
+  </si>
+  <si>
+    <t>order_RYa8RbS7hVLx2A</t>
+  </si>
+  <si>
+    <t>pay_RYa8oNcuinD0t4</t>
+  </si>
+  <si>
+    <t>dfj</t>
+  </si>
+  <si>
+    <t>567890</t>
+  </si>
+  <si>
+    <t>esi</t>
+  </si>
+  <si>
+    <t>hesi</t>
+  </si>
+  <si>
+    <t>78980</t>
+  </si>
+  <si>
+    <t>eshi</t>
+  </si>
+  <si>
+    <t>7/6/2026, 11:29:15 am</t>
+  </si>
+  <si>
+    <t>order_SydKuNSWXwR3oM</t>
+  </si>
+  <si>
+    <t>pay_SydO0QAPHmIe3d</t>
+  </si>
+  <si>
+    <t>Arsh</t>
+  </si>
+  <si>
+    <t>76879</t>
+  </si>
+  <si>
+    <t>guscvcu</t>
+  </si>
+  <si>
+    <t>gvyg</t>
+  </si>
+  <si>
+    <t>uvy</t>
+  </si>
+  <si>
+    <t>21344</t>
+  </si>
+  <si>
+    <t>rfer</t>
+  </si>
+  <si>
+    <t>7/6/2026, 11:55:52 am</t>
+  </si>
+  <si>
+    <t>order_Sydq2Y9Ae4jThr</t>
+  </si>
+  <si>
+    <t>pay_SydqADSNjTNmX5</t>
+  </si>
+  <si>
+    <t>sdf</t>
+  </si>
+  <si>
+    <t>7/6/2026, 11:59:50 am</t>
+  </si>
+  <si>
+    <t>order_Sydu9rYpedHcHI</t>
+  </si>
+  <si>
+    <t>pay_SyduJ36deF7Un4</t>
+  </si>
+  <si>
+    <t>ejvu</t>
+  </si>
+  <si>
+    <t>7/6/2026, 6:40:38 pm</t>
+  </si>
+  <si>
+    <t>order_SykjRNzId4gZGr</t>
+  </si>
+  <si>
+    <t>pay_SykjlHyqnpeAMH</t>
+  </si>
+  <si>
+    <t>54657687</t>
+  </si>
+  <si>
+    <t>eddj</t>
   </si>
 </sst>
 </file>
@@ -1737,7 +1833,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -3698,6 +3794,181 @@
         <v>3510</v>
       </c>
     </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>450</v>
+      </c>
+      <c r="B56" t="s">
+        <v>451</v>
+      </c>
+      <c r="C56" t="s">
+        <v>452</v>
+      </c>
+      <c r="D56" t="s">
+        <v>453</v>
+      </c>
+      <c r="E56" t="s">
+        <v>454</v>
+      </c>
+      <c r="F56" t="s">
+        <v>375</v>
+      </c>
+      <c r="G56" t="s">
+        <v>455</v>
+      </c>
+      <c r="H56" t="s">
+        <v>456</v>
+      </c>
+      <c r="I56" t="s">
+        <v>457</v>
+      </c>
+      <c r="J56" t="s">
+        <v>458</v>
+      </c>
+      <c r="K56">
+        <v>2760</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>459</v>
+      </c>
+      <c r="B57" t="s">
+        <v>460</v>
+      </c>
+      <c r="C57" t="s">
+        <v>461</v>
+      </c>
+      <c r="D57" t="s">
+        <v>462</v>
+      </c>
+      <c r="E57" t="s">
+        <v>463</v>
+      </c>
+      <c r="F57" t="s">
+        <v>464</v>
+      </c>
+      <c r="G57" t="s">
+        <v>465</v>
+      </c>
+      <c r="H57" t="s">
+        <v>466</v>
+      </c>
+      <c r="I57" t="s">
+        <v>467</v>
+      </c>
+      <c r="J57" t="s">
+        <v>468</v>
+      </c>
+      <c r="K57">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>469</v>
+      </c>
+      <c r="B58" t="s">
+        <v>470</v>
+      </c>
+      <c r="C58" t="s">
+        <v>471</v>
+      </c>
+      <c r="D58" t="s">
+        <v>462</v>
+      </c>
+      <c r="E58" t="s">
+        <v>463</v>
+      </c>
+      <c r="F58" t="s">
+        <v>464</v>
+      </c>
+      <c r="G58" t="s">
+        <v>465</v>
+      </c>
+      <c r="H58" t="s">
+        <v>466</v>
+      </c>
+      <c r="I58" t="s">
+        <v>467</v>
+      </c>
+      <c r="J58" t="s">
+        <v>472</v>
+      </c>
+      <c r="K58">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>473</v>
+      </c>
+      <c r="B59" t="s">
+        <v>474</v>
+      </c>
+      <c r="C59" t="s">
+        <v>475</v>
+      </c>
+      <c r="D59" t="s">
+        <v>462</v>
+      </c>
+      <c r="E59" t="s">
+        <v>463</v>
+      </c>
+      <c r="F59" t="s">
+        <v>464</v>
+      </c>
+      <c r="G59" t="s">
+        <v>465</v>
+      </c>
+      <c r="H59" t="s">
+        <v>466</v>
+      </c>
+      <c r="I59" t="s">
+        <v>467</v>
+      </c>
+      <c r="J59" t="s">
+        <v>476</v>
+      </c>
+      <c r="K59">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>477</v>
+      </c>
+      <c r="B60" t="s">
+        <v>478</v>
+      </c>
+      <c r="C60" t="s">
+        <v>479</v>
+      </c>
+      <c r="D60" t="s">
+        <v>462</v>
+      </c>
+      <c r="E60" t="s">
+        <v>480</v>
+      </c>
+      <c r="F60" t="s">
+        <v>464</v>
+      </c>
+      <c r="G60" t="s">
+        <v>465</v>
+      </c>
+      <c r="H60" t="s">
+        <v>466</v>
+      </c>
+      <c r="I60" t="s">
+        <v>467</v>
+      </c>
+      <c r="J60" t="s">
+        <v>481</v>
+      </c>
+      <c r="K60">
+        <v>290</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>